<commit_message>
feat: add v2.1.0 bulk reliability and account failover
</commit_message>
<xml_diff>
--- a/template/providers/odoo/google-sheets-template-sandbox.xlsx
+++ b/template/providers/odoo/google-sheets-template-sandbox.xlsx
@@ -2,13 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README_SETUP" sheetId="1" r:id="R27d31966da994a44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="provider" sheetId="2" r:id="R480e7a7eb3294384"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="email_list" sheetId="3" r:id="Rcd23f7c0e5c546aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="invoice_results" sheetId="4" r:id="R93eb071928aa4dbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="run_control" sheetId="5" r:id="R936c6a1a20244429"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="odoo_checklist" sheetId="6" r:id="Rdc7281bb4e6b4a8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="field_map" sheetId="7" r:id="Redcc5d45baa54b88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README_SETUP" sheetId="1" r:id="Re3a9f89bc4404253"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="provider" sheetId="2" r:id="Re20b6149ec53461d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="email_list" sheetId="3" r:id="Rdf9fa1bd72924df2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="invoice_results" sheetId="4" r:id="Ra0c9b923f9e4447d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="run_control" sheetId="5" r:id="Re9d970abbf1f4389"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="odoo_checklist" sheetId="6" r:id="R35c87982ef904f16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="field_map" sheetId="7" r:id="Rad7605816d1140b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="retry_queue" sheetId="8" r:id="R6b791e0b18794471"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="account_report" sheetId="9" r:id="Rcc919103851246c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="campaign_report" sheetId="10" r:id="Re5984bee5aef40c1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -59,7 +62,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -96,6 +99,11 @@
         <x:fgColor rgb="FFF1F5F9"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -104,7 +112,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="72">
+  <x:cellXfs count="83">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -297,6 +305,42 @@
     <x:xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -478,7 +522,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="54" t="str">
-        <x:v>InvoiceRouter v2.0.0 — Odoo Complete Bulk Email — Sandbox/Test Mode Template</x:v>
+        <x:v>InvoiceRouter v2.1.0 — Odoo Bulk Reliability — Sandbox Compatibility Workbook</x:v>
       </x:c>
       <x:c r="B1" s="55"/>
       <x:c r="C1" s="55"/>
@@ -536,7 +580,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="56" t="str">
-        <x:v>This workbook is configured for SANDBOX provider row activation. Pair it with n8n-import-workflow-sandbox-canary.json first.</x:v>
+        <x:v>Use the canonical production workflow with one enabled sandbox/test account and one recipient.</x:v>
       </x:c>
       <x:c r="B3" s="55"/>
       <x:c r="C3" s="55"/>
@@ -6184,6 +6228,62 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="81" t="str">
+        <x:v>Report_Key</x:v>
+      </x:c>
+      <x:c r="B1" s="81" t="str">
+        <x:v>Campaign_ID</x:v>
+      </x:c>
+      <x:c r="C1" s="81" t="str">
+        <x:v>Job_ID</x:v>
+      </x:c>
+      <x:c r="D1" s="81" t="str">
+        <x:v>Recipient_Email</x:v>
+      </x:c>
+      <x:c r="E1" s="81" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="F1" s="81" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G1" s="81" t="str">
+        <x:v>Sent</x:v>
+      </x:c>
+      <x:c r="H1" s="81" t="str">
+        <x:v>Queued</x:v>
+      </x:c>
+      <x:c r="I1" s="81" t="str">
+        <x:v>Failed</x:v>
+      </x:c>
+      <x:c r="J1" s="81" t="str">
+        <x:v>Manual_Review</x:v>
+      </x:c>
+      <x:c r="K1" s="81" t="str">
+        <x:v>Duplicate</x:v>
+      </x:c>
+      <x:c r="L1" s="81" t="str">
+        <x:v>Retrying</x:v>
+      </x:c>
+      <x:c r="M1" s="81" t="str">
+        <x:v>Failover</x:v>
+      </x:c>
+      <x:c r="N1" s="81" t="str">
+        <x:v>Account_ID</x:v>
+      </x:c>
+      <x:c r="O1" s="81" t="str">
+        <x:v>Updated_At</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -6208,66 +6308,99 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
-      <x:c r="A1" s="57" t="str">
+      <x:c r="A1" s="75" t="str">
         <x:v>Enabled</x:v>
       </x:c>
-      <x:c r="B1" s="57" t="str">
+      <x:c r="B1" s="75" t="str">
         <x:v>Provider</x:v>
       </x:c>
-      <x:c r="C1" s="57" t="str">
+      <x:c r="C1" s="75" t="str">
         <x:v>Account</x:v>
       </x:c>
-      <x:c r="D1" s="57" t="str">
+      <x:c r="D1" s="75" t="str">
         <x:v>Environment</x:v>
       </x:c>
-      <x:c r="E1" s="57" t="str">
+      <x:c r="E1" s="75" t="str">
         <x:v>Action</x:v>
       </x:c>
-      <x:c r="F1" s="57" t="str">
+      <x:c r="F1" s="75" t="str">
         <x:v>Method</x:v>
       </x:c>
-      <x:c r="G1" s="57" t="str">
+      <x:c r="G1" s="75" t="str">
         <x:v>Base URL</x:v>
       </x:c>
-      <x:c r="H1" s="57" t="str">
+      <x:c r="H1" s="75" t="str">
         <x:v>Endpoint</x:v>
       </x:c>
-      <x:c r="I1" s="57" t="str">
+      <x:c r="I1" s="75" t="str">
         <x:v>Auth Type</x:v>
       </x:c>
-      <x:c r="J1" s="57" t="str">
+      <x:c r="J1" s="75" t="str">
         <x:v>Username</x:v>
       </x:c>
-      <x:c r="K1" s="57" t="str">
+      <x:c r="K1" s="75" t="str">
         <x:v>Password</x:v>
       </x:c>
-      <x:c r="L1" s="57" t="str">
+      <x:c r="L1" s="75" t="str">
         <x:v>Database</x:v>
       </x:c>
-      <x:c r="M1" s="57" t="str">
+      <x:c r="M1" s="75" t="str">
         <x:v>API Key</x:v>
       </x:c>
-      <x:c r="N1" s="57" t="str">
+      <x:c r="N1" s="75" t="str">
         <x:v>API Secret</x:v>
       </x:c>
-      <x:c r="O1" s="57" t="str">
+      <x:c r="O1" s="75" t="str">
         <x:v>Extra Config JSON</x:v>
       </x:c>
-      <x:c r="P1" s="57" t="str">
+      <x:c r="P1" s="75" t="str">
         <x:v>Timeout</x:v>
       </x:c>
-      <x:c r="Q1" s="57" t="str">
+      <x:c r="Q1" s="75" t="str">
         <x:v>Notes</x:v>
       </x:c>
-      <x:c r="R1" s="55"/>
-      <x:c r="S1" s="55"/>
-      <x:c r="T1" s="55"/>
-      <x:c r="U1" s="55"/>
-      <x:c r="V1" s="55"/>
-      <x:c r="W1" s="55"/>
-      <x:c r="X1" s="55"/>
-      <x:c r="Y1" s="55"/>
-      <x:c r="Z1" s="55"/>
+      <x:c r="R1" s="80" t="str">
+        <x:v>Failover_Group</x:v>
+      </x:c>
+      <x:c r="S1" s="80" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="T1" s="80" t="str">
+        <x:v>Status_Reason</x:v>
+      </x:c>
+      <x:c r="U1" s="80" t="str">
+        <x:v>Auto_Disabled</x:v>
+      </x:c>
+      <x:c r="V1" s="80" t="str">
+        <x:v>Consecutive_Failures</x:v>
+      </x:c>
+      <x:c r="W1" s="80" t="str">
+        <x:v>Retry_Count</x:v>
+      </x:c>
+      <x:c r="X1" s="80" t="str">
+        <x:v>Cooldown_Until</x:v>
+      </x:c>
+      <x:c r="Y1" s="80" t="str">
+        <x:v>Last_Error_Type</x:v>
+      </x:c>
+      <x:c r="Z1" s="80" t="str">
+        <x:v>Last_Error</x:v>
+      </x:c>
+      <x:c r="AA1" s="81" t="str">
+        <x:v>Last_Used_At</x:v>
+      </x:c>
+      <x:c r="AB1" s="81" t="str">
+        <x:v>Total_Allocated</x:v>
+      </x:c>
+      <x:c r="AC1" s="81" t="str">
+        <x:v>Total_Sent</x:v>
+      </x:c>
+      <x:c r="AD1" s="81" t="str">
+        <x:v>Total_Failed</x:v>
+      </x:c>
+      <x:c r="AE1" s="81" t="str">
+        <x:v>Updated_At</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
       <x:c r="A2" s="66" t="b">
@@ -6306,26 +6439,47 @@
       <x:c r="L2" s="67" t="str">
         <x:v>REPLACE_ODOO_DATABASE</x:v>
       </x:c>
-      <x:c r="M2" s="67" t="str"/>
-      <x:c r="N2" s="67" t="str"/>
+      <x:c r="M2" s="67"/>
+      <x:c r="N2" s="67"/>
       <x:c r="O2" s="67" t="str">
-        <x:v>{"invoiceLifecycle":"createPostAndSendEmail","odooPostInvoice":true,"odooSendInvoiceEmail":true,"odooEmailForceSend":true,"odooEmailBody":"Your invoice has been created and posted."}</x:v>
+        <x:v>{"invoiceLifecycle":"createPostAndSendEmail","odooPostInvoice":true,"odooSendInvoiceEmail":true,"odooEmailForceSend":true}</x:v>
       </x:c>
       <x:c r="P2" s="58" t="n">
         <x:v>60</x:v>
       </x:c>
       <x:c r="Q2" s="58" t="str">
-        <x:v>SANDBOX ROW ENABLED. Replace test/sandbox credentials. Use sandbox canary workflow first, then sandbox bulk workflow.</x:v>
+        <x:v>Sandbox compatibility row</x:v>
       </x:c>
-      <x:c r="R2" s="55"/>
-      <x:c r="S2" s="55"/>
-      <x:c r="T2" s="55"/>
-      <x:c r="U2" s="55"/>
-      <x:c r="V2" s="55"/>
-      <x:c r="W2" s="55"/>
-      <x:c r="X2" s="55"/>
-      <x:c r="Y2" s="55"/>
-      <x:c r="Z2" s="55"/>
+      <x:c r="R2" s="55" t="str">
+        <x:v>odoo-sandbox</x:v>
+      </x:c>
+      <x:c r="S2" s="55" t="str">
+        <x:v>READY</x:v>
+      </x:c>
+      <x:c r="T2" s="55" t="str"/>
+      <x:c r="U2" s="72" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V2" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W2" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X2" s="55" t="str"/>
+      <x:c r="Y2" s="55" t="str"/>
+      <x:c r="Z2" s="55" t="str"/>
+      <x:c r="AA2" t="str"/>
+      <x:c r="AB2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AC2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AD2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE2" t="str"/>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
       <x:c r="A3" s="66" t="b">
@@ -6335,7 +6489,7 @@
         <x:v>Odoo</x:v>
       </x:c>
       <x:c r="C3" s="58" t="str">
-        <x:v>Odoo Live Canary</x:v>
+        <x:v>Odoo Live Primary</x:v>
       </x:c>
       <x:c r="D3" s="58" t="str">
         <x:v>live</x:v>
@@ -6364,26 +6518,47 @@
       <x:c r="L3" s="67" t="str">
         <x:v>REPLACE_ODOO_DATABASE</x:v>
       </x:c>
-      <x:c r="M3" s="67" t="str"/>
-      <x:c r="N3" s="67" t="str"/>
+      <x:c r="M3" s="67"/>
+      <x:c r="N3" s="67"/>
       <x:c r="O3" s="67" t="str">
-        <x:v>{"invoiceLifecycle":"createPostAndSendEmail","odooPostInvoice":true,"odooSendInvoiceEmail":true,"odooEmailForceSend":true,"odooEmailBody":"Your invoice has been created and posted."}</x:v>
+        <x:v>{"invoiceLifecycle":"createPostAndSendEmail","odooPostInvoice":true,"odooSendInvoiceEmail":true,"odooEmailForceSend":true}</x:v>
       </x:c>
       <x:c r="P3" s="58" t="n">
         <x:v>60</x:v>
       </x:c>
       <x:c r="Q3" s="58" t="str">
-        <x:v>LIVE ROW DISABLED in this workbook. Use google-sheets-template-live.xlsx for live mode.</x:v>
+        <x:v>Disabled in sandbox workbook</x:v>
       </x:c>
-      <x:c r="R3" s="55"/>
-      <x:c r="S3" s="55"/>
-      <x:c r="T3" s="55"/>
-      <x:c r="U3" s="55"/>
-      <x:c r="V3" s="55"/>
-      <x:c r="W3" s="55"/>
-      <x:c r="X3" s="55"/>
-      <x:c r="Y3" s="55"/>
-      <x:c r="Z3" s="55"/>
+      <x:c r="R3" s="55" t="str">
+        <x:v>odoo-production</x:v>
+      </x:c>
+      <x:c r="S3" s="55" t="str">
+        <x:v>DISABLED_USER</x:v>
+      </x:c>
+      <x:c r="T3" s="55" t="str"/>
+      <x:c r="U3" s="72" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V3" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W3" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X3" s="55" t="str"/>
+      <x:c r="Y3" s="55" t="str"/>
+      <x:c r="Z3" s="55" t="str"/>
+      <x:c r="AA3" t="str"/>
+      <x:c r="AB3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AC3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AD3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE3" t="str"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="55"/>
@@ -11930,22 +12105,36 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="57" t="str">
+      <x:c r="A1" s="75" t="str">
         <x:v>Email</x:v>
       </x:c>
-      <x:c r="B1" s="57" t="str">
+      <x:c r="B1" s="75" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="C1" s="75" t="str">
         <x:v>Name</x:v>
       </x:c>
-      <x:c r="C1" s="57" t="str">
+      <x:c r="D1" s="80" t="str">
         <x:v>Address</x:v>
       </x:c>
-      <x:c r="D1" s="55"/>
-      <x:c r="E1" s="55"/>
-      <x:c r="F1" s="55"/>
-      <x:c r="G1" s="55"/>
-      <x:c r="H1" s="55"/>
-      <x:c r="I1" s="55"/>
-      <x:c r="J1" s="55"/>
+      <x:c r="E1" s="80" t="str">
+        <x:v>Job_ID</x:v>
+      </x:c>
+      <x:c r="F1" s="80" t="str">
+        <x:v>Campaign_ID</x:v>
+      </x:c>
+      <x:c r="G1" s="80" t="str">
+        <x:v>Attempt_Count</x:v>
+      </x:c>
+      <x:c r="H1" s="80" t="str">
+        <x:v>Last_Account</x:v>
+      </x:c>
+      <x:c r="I1" s="80" t="str">
+        <x:v>Last_Error</x:v>
+      </x:c>
+      <x:c r="J1" s="80" t="str">
+        <x:v>Updated_At</x:v>
+      </x:c>
       <x:c r="K1" s="55"/>
       <x:c r="L1" s="55"/>
       <x:c r="M1" s="55"/>
@@ -11965,19 +12154,25 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="67" t="str">
-        <x:v>victorsteele428@gmail.com</x:v>
+        <x:v>customer@example.com</x:v>
       </x:c>
       <x:c r="B2" s="70" t="str">
-        <x:v>Victor Steele</x:v>
+        <x:v>PENDING</x:v>
       </x:c>
-      <x:c r="C2" s="70" t="str"/>
-      <x:c r="D2" s="55"/>
-      <x:c r="E2" s="55"/>
-      <x:c r="F2" s="55"/>
-      <x:c r="G2" s="55"/>
-      <x:c r="H2" s="55"/>
-      <x:c r="I2" s="55"/>
-      <x:c r="J2" s="55"/>
+      <x:c r="C2" s="70" t="str">
+        <x:v>Customer Example</x:v>
+      </x:c>
+      <x:c r="D2" s="55" t="str"/>
+      <x:c r="E2" s="55" t="str"/>
+      <x:c r="F2" s="55" t="str">
+        <x:v>sandbox-campaign-001</x:v>
+      </x:c>
+      <x:c r="G2" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H2" s="55" t="str"/>
+      <x:c r="I2" s="55" t="str"/>
+      <x:c r="J2" s="55" t="str"/>
       <x:c r="K2" s="55"/>
       <x:c r="L2" s="55"/>
       <x:c r="M2" s="55"/>
@@ -11999,15 +12194,21 @@
       <x:c r="A3" s="67" t="str">
         <x:v>customer2@example.com</x:v>
       </x:c>
-      <x:c r="B3" s="70" t="str"/>
+      <x:c r="B3" s="70" t="str">
+        <x:v>PENDING</x:v>
+      </x:c>
       <x:c r="C3" s="70" t="str"/>
-      <x:c r="D3" s="55"/>
-      <x:c r="E3" s="55"/>
-      <x:c r="F3" s="55"/>
-      <x:c r="G3" s="55"/>
-      <x:c r="H3" s="55"/>
-      <x:c r="I3" s="55"/>
-      <x:c r="J3" s="55"/>
+      <x:c r="D3" s="55" t="str"/>
+      <x:c r="E3" s="55" t="str"/>
+      <x:c r="F3" s="55" t="str">
+        <x:v>sandbox-campaign-001</x:v>
+      </x:c>
+      <x:c r="G3" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H3" s="55" t="str"/>
+      <x:c r="I3" s="55" t="str"/>
+      <x:c r="J3" s="55" t="str"/>
       <x:c r="K3" s="55"/>
       <x:c r="L3" s="55"/>
       <x:c r="M3" s="55"/>
@@ -12029,15 +12230,21 @@
       <x:c r="A4" s="67" t="str">
         <x:v>customer3@example.com</x:v>
       </x:c>
-      <x:c r="B4" s="70" t="str"/>
+      <x:c r="B4" s="70" t="str">
+        <x:v>PENDING</x:v>
+      </x:c>
       <x:c r="C4" s="70" t="str"/>
-      <x:c r="D4" s="55"/>
-      <x:c r="E4" s="55"/>
-      <x:c r="F4" s="55"/>
-      <x:c r="G4" s="55"/>
-      <x:c r="H4" s="55"/>
-      <x:c r="I4" s="55"/>
-      <x:c r="J4" s="55"/>
+      <x:c r="D4" s="55" t="str"/>
+      <x:c r="E4" s="55" t="str"/>
+      <x:c r="F4" s="55" t="str">
+        <x:v>sandbox-campaign-001</x:v>
+      </x:c>
+      <x:c r="G4" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H4" s="55" t="str"/>
+      <x:c r="I4" s="55" t="str"/>
+      <x:c r="J4" s="55" t="str"/>
       <x:c r="K4" s="55"/>
       <x:c r="L4" s="55"/>
       <x:c r="M4" s="55"/>
@@ -17584,197 +17791,230 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="50" customHeight="1">
-      <x:c r="A1" s="57" t="str">
+      <x:c r="A1" s="75" t="str">
         <x:v>writeback_key</x:v>
       </x:c>
-      <x:c r="B1" s="57" t="str">
+      <x:c r="B1" s="75" t="str">
         <x:v>writeback_action</x:v>
       </x:c>
-      <x:c r="C1" s="57" t="str">
+      <x:c r="C1" s="75" t="str">
         <x:v>writeback_target</x:v>
       </x:c>
-      <x:c r="D1" s="57" t="str">
+      <x:c r="D1" s="75" t="str">
         <x:v>key_mode</x:v>
       </x:c>
-      <x:c r="E1" s="57" t="str">
+      <x:c r="E1" s="75" t="str">
         <x:v>request_id</x:v>
       </x:c>
-      <x:c r="F1" s="57" t="str">
+      <x:c r="F1" s="75" t="str">
         <x:v>transaction_id</x:v>
       </x:c>
-      <x:c r="G1" s="57" t="str">
+      <x:c r="G1" s="75" t="str">
         <x:v>idempotency_key</x:v>
       </x:c>
-      <x:c r="H1" s="57" t="str">
+      <x:c r="H1" s="75" t="str">
+        <x:v>job_id</x:v>
+      </x:c>
+      <x:c r="I1" s="75" t="str">
+        <x:v>campaign_id</x:v>
+      </x:c>
+      <x:c r="J1" s="75" t="str">
         <x:v>provider_id</x:v>
       </x:c>
-      <x:c r="I1" s="57" t="str">
+      <x:c r="K1" s="75" t="str">
         <x:v>profile_id</x:v>
       </x:c>
-      <x:c r="J1" s="57" t="str">
+      <x:c r="L1" s="75" t="str">
         <x:v>account_id</x:v>
       </x:c>
-      <x:c r="K1" s="57" t="str">
+      <x:c r="M1" s="75" t="str">
         <x:v>action_id</x:v>
       </x:c>
-      <x:c r="L1" s="57" t="str">
+      <x:c r="N1" s="75" t="str">
         <x:v>worker_id</x:v>
       </x:c>
-      <x:c r="M1" s="57" t="str">
+      <x:c r="O1" s="75" t="str">
         <x:v>recipient_email</x:v>
       </x:c>
-      <x:c r="N1" s="57" t="str">
+      <x:c r="P1" s="75" t="str">
         <x:v>workflow_state</x:v>
       </x:c>
-      <x:c r="O1" s="57" t="str">
+      <x:c r="Q1" s="75" t="str">
         <x:v>result</x:v>
       </x:c>
-      <x:c r="P1" s="57" t="str">
+      <x:c r="R1" s="75" t="str">
         <x:v>invoice_status</x:v>
       </x:c>
-      <x:c r="Q1" s="57" t="str">
+      <x:c r="S1" s="75" t="str">
         <x:v>provider_status</x:v>
       </x:c>
-      <x:c r="R1" s="57" t="str">
+      <x:c r="T1" s="75" t="str">
         <x:v>transport_status</x:v>
       </x:c>
-      <x:c r="S1" s="57" t="str">
+      <x:c r="U1" s="75" t="str">
         <x:v>provider_customer_id</x:v>
       </x:c>
-      <x:c r="T1" s="57" t="str">
+      <x:c r="V1" s="75" t="str">
         <x:v>customer_status</x:v>
       </x:c>
-      <x:c r="U1" s="57" t="str">
+      <x:c r="W1" s="75" t="str">
         <x:v>post_status</x:v>
       </x:c>
-      <x:c r="V1" s="57" t="str">
+      <x:c r="X1" s="75" t="str">
         <x:v>email_send_requested</x:v>
       </x:c>
-      <x:c r="W1" s="57" t="str">
+      <x:c r="Y1" s="75" t="str">
         <x:v>email_send_status</x:v>
       </x:c>
-      <x:c r="X1" s="57" t="str">
+      <x:c r="Z1" s="75" t="str">
         <x:v>email_send_method</x:v>
       </x:c>
-      <x:c r="Y1" s="57" t="str">
+      <x:c r="AA1" s="82" t="str">
         <x:v>email_error_message</x:v>
       </x:c>
-      <x:c r="Z1" s="57" t="str">
+      <x:c r="AB1" s="82" t="str">
+        <x:v>email_evidence</x:v>
+      </x:c>
+      <x:c r="AC1" s="82" t="str">
+        <x:v>lifecycle_outcome</x:v>
+      </x:c>
+      <x:c r="AD1" s="82" t="str">
+        <x:v>lifecycle_failed_step</x:v>
+      </x:c>
+      <x:c r="AE1" s="82" t="str">
+        <x:v>lifecycle_checkpoint</x:v>
+      </x:c>
+      <x:c r="AF1" s="82" t="str">
+        <x:v>retry_resume_stage</x:v>
+      </x:c>
+      <x:c r="AG1" s="82" t="str">
+        <x:v>retry_resume</x:v>
+      </x:c>
+      <x:c r="AH1" s="82" t="str">
         <x:v>provider_invoice_id</x:v>
       </x:c>
-      <x:c r="AA1" s="20" t="str">
+      <x:c r="AI1" s="82" t="str">
         <x:v>invoice_number</x:v>
       </x:c>
-      <x:c r="AB1" s="20" t="str">
+      <x:c r="AJ1" s="82" t="str">
         <x:v>invoice_url</x:v>
       </x:c>
-      <x:c r="AC1" s="20" t="str">
+      <x:c r="AK1" s="82" t="str">
         <x:v>pdf_url</x:v>
       </x:c>
-      <x:c r="AD1" s="20" t="str">
+      <x:c r="AL1" s="82" t="str">
         <x:v>http_status</x:v>
       </x:c>
-      <x:c r="AE1" s="20" t="str">
+      <x:c r="AM1" s="82" t="str">
         <x:v>error_type</x:v>
       </x:c>
-      <x:c r="AF1" s="20" t="str">
+      <x:c r="AN1" s="82" t="str">
         <x:v>error_category</x:v>
       </x:c>
-      <x:c r="AG1" s="20" t="str">
+      <x:c r="AO1" s="82" t="str">
         <x:v>error_severity</x:v>
       </x:c>
-      <x:c r="AH1" s="20" t="str">
+      <x:c r="AP1" s="82" t="str">
         <x:v>error_code</x:v>
       </x:c>
-      <x:c r="AI1" s="20" t="str">
+      <x:c r="AQ1" s="82" t="str">
         <x:v>error_message</x:v>
       </x:c>
-      <x:c r="AJ1" s="20" t="str">
+      <x:c r="AR1" s="82" t="str">
         <x:v>retry_scheduled</x:v>
       </x:c>
-      <x:c r="AK1" s="20" t="str">
+      <x:c r="AS1" s="82" t="str">
         <x:v>retry_count</x:v>
       </x:c>
-      <x:c r="AL1" s="20" t="str">
+      <x:c r="AT1" s="82" t="str">
         <x:v>retry_delay_seconds</x:v>
       </x:c>
-      <x:c r="AM1" s="20" t="str">
+      <x:c r="AU1" s="82" t="str">
         <x:v>retry_decision_source</x:v>
       </x:c>
-      <x:c r="AN1" s="20" t="str">
+      <x:c r="AV1" s="82" t="str">
         <x:v>retry_decision_reason</x:v>
       </x:c>
-      <x:c r="AO1" s="20" t="str">
+      <x:c r="AW1" s="82" t="str">
         <x:v>retry_after_seconds</x:v>
       </x:c>
-      <x:c r="AP1" s="20" t="str">
+      <x:c r="AX1" s="82" t="str">
         <x:v>retry_delay_hint_seconds</x:v>
       </x:c>
-      <x:c r="AQ1" s="20" t="str">
+      <x:c r="AY1" s="82" t="str">
         <x:v>next_retry_at</x:v>
       </x:c>
-      <x:c r="AR1" s="20" t="str">
+      <x:c r="AZ1" s="82" t="str">
         <x:v>lifecycle_mode</x:v>
       </x:c>
-      <x:c r="AS1" s="20" t="str">
+      <x:c r="BA1" s="82" t="str">
         <x:v>lifecycle_steps</x:v>
       </x:c>
-      <x:c r="AT1" s="20" t="str">
+      <x:c r="BB1" s="82" t="str">
         <x:v>provider_recipe_id</x:v>
       </x:c>
-      <x:c r="AU1" s="20" t="str">
+      <x:c r="BC1" s="82" t="str">
         <x:v>preset_self_check_mode</x:v>
       </x:c>
-      <x:c r="AV1" s="20" t="str">
+      <x:c r="BD1" s="82" t="str">
         <x:v>preset_self_check_approved</x:v>
       </x:c>
-      <x:c r="AW1" s="20" t="str">
+      <x:c r="BE1" s="82" t="str">
         <x:v>preset_self_check</x:v>
       </x:c>
-      <x:c r="AX1" s="20" t="str">
+      <x:c r="BF1" s="82" t="str">
         <x:v>activation_mode</x:v>
       </x:c>
-      <x:c r="AY1" s="20" t="str">
+      <x:c r="BG1" s="82" t="str">
         <x:v>activation_approved</x:v>
       </x:c>
-      <x:c r="AZ1" s="20" t="str">
+      <x:c r="BH1" s="82" t="str">
         <x:v>activation_safety</x:v>
       </x:c>
-      <x:c r="BA1" s="20" t="str">
+      <x:c r="BI1" s="82" t="str">
         <x:v>bulk_run_id</x:v>
       </x:c>
-      <x:c r="BB1" s="20" t="str">
+      <x:c r="BJ1" s="82" t="str">
         <x:v>bulk_item_number</x:v>
       </x:c>
-      <x:c r="BC1" s="20" t="str">
+      <x:c r="BK1" s="82" t="str">
         <x:v>bulk_total_items</x:v>
       </x:c>
-      <x:c r="BD1" s="20" t="str">
+      <x:c r="BL1" s="82" t="str">
         <x:v>bulk_decision</x:v>
       </x:c>
-      <x:c r="BE1" s="20" t="str">
+      <x:c r="BM1" s="81" t="str">
         <x:v>bulk_safety</x:v>
       </x:c>
-      <x:c r="BF1" s="20" t="str">
+      <x:c r="BN1" s="81" t="str">
         <x:v>bulk_summary</x:v>
       </x:c>
-      <x:c r="BG1" s="20" t="str">
+      <x:c r="BO1" s="81" t="str">
         <x:v>retryable_by_policy</x:v>
       </x:c>
-      <x:c r="BH1" s="20" t="str">
+      <x:c r="BP1" s="81" t="str">
         <x:v>non_retryable_by_policy</x:v>
       </x:c>
-      <x:c r="BI1" s="20" t="str">
+      <x:c r="BQ1" s="81" t="str">
         <x:v>duplicate_prevention</x:v>
       </x:c>
-      <x:c r="BJ1" s="20" t="str">
+      <x:c r="BR1" s="81" t="str">
         <x:v>checked_at</x:v>
       </x:c>
-      <x:c r="BK1" s="20" t="str">
+      <x:c r="BS1" s="81" t="str">
         <x:v>managed_at</x:v>
       </x:c>
-      <x:c r="BL1" s="20" t="str">
+      <x:c r="BT1" s="81" t="str">
         <x:v>updated_at</x:v>
+      </x:c>
+      <x:c r="BU1" s="81" t="str">
+        <x:v>failover_scheduled</x:v>
+      </x:c>
+      <x:c r="BV1" s="81" t="str">
+        <x:v>recipient_status</x:v>
+      </x:c>
+      <x:c r="BW1" s="81" t="str">
+        <x:v>provider_operational_status</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -34795,7 +35035,7 @@
         <x:v>Odoo base domain without trailing slash</x:v>
       </x:c>
       <x:c r="E2" s="58" t="str">
-        <x:v>https://apple-zone1.odoo.com</x:v>
+        <x:v>https://YOUR-SUBDOMAIN.odoo.com</x:v>
       </x:c>
       <x:c r="F2" s="55"/>
       <x:c r="G2" s="55"/>
@@ -34947,7 +35187,7 @@
         <x:v>Exact Odoo database technical name</x:v>
       </x:c>
       <x:c r="E6" s="58" t="str">
-        <x:v>apple-zone1</x:v>
+        <x:v>YOUR_ODOO_DATABASE</x:v>
       </x:c>
       <x:c r="F6" s="55"/>
       <x:c r="G6" s="55"/>
@@ -40446,4 +40686,155 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="81" t="str">
+        <x:v>Job_ID</x:v>
+      </x:c>
+      <x:c r="B1" s="81" t="str">
+        <x:v>Campaign_ID</x:v>
+      </x:c>
+      <x:c r="C1" s="81" t="str">
+        <x:v>Recipient_Email</x:v>
+      </x:c>
+      <x:c r="D1" s="81" t="str">
+        <x:v>Original_Profile_ID</x:v>
+      </x:c>
+      <x:c r="E1" s="81" t="str">
+        <x:v>Current_Profile_ID</x:v>
+      </x:c>
+      <x:c r="F1" s="81" t="str">
+        <x:v>Attempted_Profile_IDs</x:v>
+      </x:c>
+      <x:c r="G1" s="81" t="str">
+        <x:v>Failover_Group</x:v>
+      </x:c>
+      <x:c r="H1" s="81" t="str">
+        <x:v>Side_Effect_Stage</x:v>
+      </x:c>
+      <x:c r="I1" s="81" t="str">
+        <x:v>Required_Profile_ID</x:v>
+      </x:c>
+      <x:c r="J1" s="81" t="str">
+        <x:v>Provider_Invoice_ID</x:v>
+      </x:c>
+      <x:c r="K1" s="81" t="str">
+        <x:v>Lifecycle_Checkpoint</x:v>
+      </x:c>
+      <x:c r="L1" s="81" t="str">
+        <x:v>Resume_Stage</x:v>
+      </x:c>
+      <x:c r="M1" s="81" t="str">
+        <x:v>Retry_Count</x:v>
+      </x:c>
+      <x:c r="N1" s="81" t="str">
+        <x:v>Failover_Count</x:v>
+      </x:c>
+      <x:c r="O1" s="81" t="str">
+        <x:v>Next_Retry_At</x:v>
+      </x:c>
+      <x:c r="P1" s="81" t="str">
+        <x:v>Last_Error_Type</x:v>
+      </x:c>
+      <x:c r="Q1" s="81" t="str">
+        <x:v>Last_Error</x:v>
+      </x:c>
+      <x:c r="R1" s="81" t="str">
+        <x:v>Queue_Status</x:v>
+      </x:c>
+      <x:c r="S1" s="81" t="str">
+        <x:v>Updated_At</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="81" t="str">
+        <x:v>Report_Key</x:v>
+      </x:c>
+      <x:c r="B1" s="81" t="str">
+        <x:v>Campaign_ID</x:v>
+      </x:c>
+      <x:c r="C1" s="81" t="str">
+        <x:v>Provider</x:v>
+      </x:c>
+      <x:c r="D1" s="81" t="str">
+        <x:v>Account_ID</x:v>
+      </x:c>
+      <x:c r="E1" s="81" t="str">
+        <x:v>Account_Name</x:v>
+      </x:c>
+      <x:c r="F1" s="81" t="str">
+        <x:v>Profile_ID</x:v>
+      </x:c>
+      <x:c r="G1" s="81" t="str">
+        <x:v>Current_Status</x:v>
+      </x:c>
+      <x:c r="H1" s="81" t="str">
+        <x:v>Enabled</x:v>
+      </x:c>
+      <x:c r="I1" s="81" t="str">
+        <x:v>Allocated</x:v>
+      </x:c>
+      <x:c r="J1" s="81" t="str">
+        <x:v>Attempted</x:v>
+      </x:c>
+      <x:c r="K1" s="81" t="str">
+        <x:v>Succeeded</x:v>
+      </x:c>
+      <x:c r="L1" s="81" t="str">
+        <x:v>Email_Sent</x:v>
+      </x:c>
+      <x:c r="M1" s="81" t="str">
+        <x:v>Email_Queued</x:v>
+      </x:c>
+      <x:c r="N1" s="81" t="str">
+        <x:v>Failed</x:v>
+      </x:c>
+      <x:c r="O1" s="81" t="str">
+        <x:v>Retried</x:v>
+      </x:c>
+      <x:c r="P1" s="81" t="str">
+        <x:v>Failover_Count</x:v>
+      </x:c>
+      <x:c r="Q1" s="81" t="str">
+        <x:v>Failover_From</x:v>
+      </x:c>
+      <x:c r="R1" s="81" t="str">
+        <x:v>Failover_To</x:v>
+      </x:c>
+      <x:c r="S1" s="81" t="str">
+        <x:v>Auto_Disabled</x:v>
+      </x:c>
+      <x:c r="T1" s="81" t="str">
+        <x:v>Disabled_Reason</x:v>
+      </x:c>
+      <x:c r="U1" s="81" t="str">
+        <x:v>Last_Error_Type</x:v>
+      </x:c>
+      <x:c r="V1" s="81" t="str">
+        <x:v>Last_Error</x:v>
+      </x:c>
+      <x:c r="W1" s="81" t="str">
+        <x:v>Last_Used_At</x:v>
+      </x:c>
+      <x:c r="X1" s="81" t="str">
+        <x:v>Updated_At</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add v2.1.0 bulk reliability and account failover (#8)
</commit_message>
<xml_diff>
--- a/template/providers/odoo/google-sheets-template-sandbox.xlsx
+++ b/template/providers/odoo/google-sheets-template-sandbox.xlsx
@@ -2,13 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README_SETUP" sheetId="1" r:id="R27d31966da994a44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="provider" sheetId="2" r:id="R480e7a7eb3294384"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="email_list" sheetId="3" r:id="Rcd23f7c0e5c546aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="invoice_results" sheetId="4" r:id="R93eb071928aa4dbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="run_control" sheetId="5" r:id="R936c6a1a20244429"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="odoo_checklist" sheetId="6" r:id="Rdc7281bb4e6b4a8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="field_map" sheetId="7" r:id="Redcc5d45baa54b88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README_SETUP" sheetId="1" r:id="Re3a9f89bc4404253"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="provider" sheetId="2" r:id="Re20b6149ec53461d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="email_list" sheetId="3" r:id="Rdf9fa1bd72924df2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="invoice_results" sheetId="4" r:id="Ra0c9b923f9e4447d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="run_control" sheetId="5" r:id="Re9d970abbf1f4389"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="odoo_checklist" sheetId="6" r:id="R35c87982ef904f16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="field_map" sheetId="7" r:id="Rad7605816d1140b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="retry_queue" sheetId="8" r:id="R6b791e0b18794471"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="account_report" sheetId="9" r:id="Rcc919103851246c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="campaign_report" sheetId="10" r:id="Re5984bee5aef40c1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -59,7 +62,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -96,6 +99,11 @@
         <x:fgColor rgb="FFF1F5F9"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -104,7 +112,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="72">
+  <x:cellXfs count="83">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -297,6 +305,42 @@
     <x:xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -478,7 +522,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="54" t="str">
-        <x:v>InvoiceRouter v2.0.0 — Odoo Complete Bulk Email — Sandbox/Test Mode Template</x:v>
+        <x:v>InvoiceRouter v2.1.0 — Odoo Bulk Reliability — Sandbox Compatibility Workbook</x:v>
       </x:c>
       <x:c r="B1" s="55"/>
       <x:c r="C1" s="55"/>
@@ -536,7 +580,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="56" t="str">
-        <x:v>This workbook is configured for SANDBOX provider row activation. Pair it with n8n-import-workflow-sandbox-canary.json first.</x:v>
+        <x:v>Use the canonical production workflow with one enabled sandbox/test account and one recipient.</x:v>
       </x:c>
       <x:c r="B3" s="55"/>
       <x:c r="C3" s="55"/>
@@ -6184,6 +6228,62 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="81" t="str">
+        <x:v>Report_Key</x:v>
+      </x:c>
+      <x:c r="B1" s="81" t="str">
+        <x:v>Campaign_ID</x:v>
+      </x:c>
+      <x:c r="C1" s="81" t="str">
+        <x:v>Job_ID</x:v>
+      </x:c>
+      <x:c r="D1" s="81" t="str">
+        <x:v>Recipient_Email</x:v>
+      </x:c>
+      <x:c r="E1" s="81" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="F1" s="81" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="G1" s="81" t="str">
+        <x:v>Sent</x:v>
+      </x:c>
+      <x:c r="H1" s="81" t="str">
+        <x:v>Queued</x:v>
+      </x:c>
+      <x:c r="I1" s="81" t="str">
+        <x:v>Failed</x:v>
+      </x:c>
+      <x:c r="J1" s="81" t="str">
+        <x:v>Manual_Review</x:v>
+      </x:c>
+      <x:c r="K1" s="81" t="str">
+        <x:v>Duplicate</x:v>
+      </x:c>
+      <x:c r="L1" s="81" t="str">
+        <x:v>Retrying</x:v>
+      </x:c>
+      <x:c r="M1" s="81" t="str">
+        <x:v>Failover</x:v>
+      </x:c>
+      <x:c r="N1" s="81" t="str">
+        <x:v>Account_ID</x:v>
+      </x:c>
+      <x:c r="O1" s="81" t="str">
+        <x:v>Updated_At</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -6208,66 +6308,99 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
-      <x:c r="A1" s="57" t="str">
+      <x:c r="A1" s="75" t="str">
         <x:v>Enabled</x:v>
       </x:c>
-      <x:c r="B1" s="57" t="str">
+      <x:c r="B1" s="75" t="str">
         <x:v>Provider</x:v>
       </x:c>
-      <x:c r="C1" s="57" t="str">
+      <x:c r="C1" s="75" t="str">
         <x:v>Account</x:v>
       </x:c>
-      <x:c r="D1" s="57" t="str">
+      <x:c r="D1" s="75" t="str">
         <x:v>Environment</x:v>
       </x:c>
-      <x:c r="E1" s="57" t="str">
+      <x:c r="E1" s="75" t="str">
         <x:v>Action</x:v>
       </x:c>
-      <x:c r="F1" s="57" t="str">
+      <x:c r="F1" s="75" t="str">
         <x:v>Method</x:v>
       </x:c>
-      <x:c r="G1" s="57" t="str">
+      <x:c r="G1" s="75" t="str">
         <x:v>Base URL</x:v>
       </x:c>
-      <x:c r="H1" s="57" t="str">
+      <x:c r="H1" s="75" t="str">
         <x:v>Endpoint</x:v>
       </x:c>
-      <x:c r="I1" s="57" t="str">
+      <x:c r="I1" s="75" t="str">
         <x:v>Auth Type</x:v>
       </x:c>
-      <x:c r="J1" s="57" t="str">
+      <x:c r="J1" s="75" t="str">
         <x:v>Username</x:v>
       </x:c>
-      <x:c r="K1" s="57" t="str">
+      <x:c r="K1" s="75" t="str">
         <x:v>Password</x:v>
       </x:c>
-      <x:c r="L1" s="57" t="str">
+      <x:c r="L1" s="75" t="str">
         <x:v>Database</x:v>
       </x:c>
-      <x:c r="M1" s="57" t="str">
+      <x:c r="M1" s="75" t="str">
         <x:v>API Key</x:v>
       </x:c>
-      <x:c r="N1" s="57" t="str">
+      <x:c r="N1" s="75" t="str">
         <x:v>API Secret</x:v>
       </x:c>
-      <x:c r="O1" s="57" t="str">
+      <x:c r="O1" s="75" t="str">
         <x:v>Extra Config JSON</x:v>
       </x:c>
-      <x:c r="P1" s="57" t="str">
+      <x:c r="P1" s="75" t="str">
         <x:v>Timeout</x:v>
       </x:c>
-      <x:c r="Q1" s="57" t="str">
+      <x:c r="Q1" s="75" t="str">
         <x:v>Notes</x:v>
       </x:c>
-      <x:c r="R1" s="55"/>
-      <x:c r="S1" s="55"/>
-      <x:c r="T1" s="55"/>
-      <x:c r="U1" s="55"/>
-      <x:c r="V1" s="55"/>
-      <x:c r="W1" s="55"/>
-      <x:c r="X1" s="55"/>
-      <x:c r="Y1" s="55"/>
-      <x:c r="Z1" s="55"/>
+      <x:c r="R1" s="80" t="str">
+        <x:v>Failover_Group</x:v>
+      </x:c>
+      <x:c r="S1" s="80" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="T1" s="80" t="str">
+        <x:v>Status_Reason</x:v>
+      </x:c>
+      <x:c r="U1" s="80" t="str">
+        <x:v>Auto_Disabled</x:v>
+      </x:c>
+      <x:c r="V1" s="80" t="str">
+        <x:v>Consecutive_Failures</x:v>
+      </x:c>
+      <x:c r="W1" s="80" t="str">
+        <x:v>Retry_Count</x:v>
+      </x:c>
+      <x:c r="X1" s="80" t="str">
+        <x:v>Cooldown_Until</x:v>
+      </x:c>
+      <x:c r="Y1" s="80" t="str">
+        <x:v>Last_Error_Type</x:v>
+      </x:c>
+      <x:c r="Z1" s="80" t="str">
+        <x:v>Last_Error</x:v>
+      </x:c>
+      <x:c r="AA1" s="81" t="str">
+        <x:v>Last_Used_At</x:v>
+      </x:c>
+      <x:c r="AB1" s="81" t="str">
+        <x:v>Total_Allocated</x:v>
+      </x:c>
+      <x:c r="AC1" s="81" t="str">
+        <x:v>Total_Sent</x:v>
+      </x:c>
+      <x:c r="AD1" s="81" t="str">
+        <x:v>Total_Failed</x:v>
+      </x:c>
+      <x:c r="AE1" s="81" t="str">
+        <x:v>Updated_At</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
       <x:c r="A2" s="66" t="b">
@@ -6306,26 +6439,47 @@
       <x:c r="L2" s="67" t="str">
         <x:v>REPLACE_ODOO_DATABASE</x:v>
       </x:c>
-      <x:c r="M2" s="67" t="str"/>
-      <x:c r="N2" s="67" t="str"/>
+      <x:c r="M2" s="67"/>
+      <x:c r="N2" s="67"/>
       <x:c r="O2" s="67" t="str">
-        <x:v>{"invoiceLifecycle":"createPostAndSendEmail","odooPostInvoice":true,"odooSendInvoiceEmail":true,"odooEmailForceSend":true,"odooEmailBody":"Your invoice has been created and posted."}</x:v>
+        <x:v>{"invoiceLifecycle":"createPostAndSendEmail","odooPostInvoice":true,"odooSendInvoiceEmail":true,"odooEmailForceSend":true}</x:v>
       </x:c>
       <x:c r="P2" s="58" t="n">
         <x:v>60</x:v>
       </x:c>
       <x:c r="Q2" s="58" t="str">
-        <x:v>SANDBOX ROW ENABLED. Replace test/sandbox credentials. Use sandbox canary workflow first, then sandbox bulk workflow.</x:v>
+        <x:v>Sandbox compatibility row</x:v>
       </x:c>
-      <x:c r="R2" s="55"/>
-      <x:c r="S2" s="55"/>
-      <x:c r="T2" s="55"/>
-      <x:c r="U2" s="55"/>
-      <x:c r="V2" s="55"/>
-      <x:c r="W2" s="55"/>
-      <x:c r="X2" s="55"/>
-      <x:c r="Y2" s="55"/>
-      <x:c r="Z2" s="55"/>
+      <x:c r="R2" s="55" t="str">
+        <x:v>odoo-sandbox</x:v>
+      </x:c>
+      <x:c r="S2" s="55" t="str">
+        <x:v>READY</x:v>
+      </x:c>
+      <x:c r="T2" s="55" t="str"/>
+      <x:c r="U2" s="72" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V2" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W2" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X2" s="55" t="str"/>
+      <x:c r="Y2" s="55" t="str"/>
+      <x:c r="Z2" s="55" t="str"/>
+      <x:c r="AA2" t="str"/>
+      <x:c r="AB2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AC2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AD2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE2" t="str"/>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
       <x:c r="A3" s="66" t="b">
@@ -6335,7 +6489,7 @@
         <x:v>Odoo</x:v>
       </x:c>
       <x:c r="C3" s="58" t="str">
-        <x:v>Odoo Live Canary</x:v>
+        <x:v>Odoo Live Primary</x:v>
       </x:c>
       <x:c r="D3" s="58" t="str">
         <x:v>live</x:v>
@@ -6364,26 +6518,47 @@
       <x:c r="L3" s="67" t="str">
         <x:v>REPLACE_ODOO_DATABASE</x:v>
       </x:c>
-      <x:c r="M3" s="67" t="str"/>
-      <x:c r="N3" s="67" t="str"/>
+      <x:c r="M3" s="67"/>
+      <x:c r="N3" s="67"/>
       <x:c r="O3" s="67" t="str">
-        <x:v>{"invoiceLifecycle":"createPostAndSendEmail","odooPostInvoice":true,"odooSendInvoiceEmail":true,"odooEmailForceSend":true,"odooEmailBody":"Your invoice has been created and posted."}</x:v>
+        <x:v>{"invoiceLifecycle":"createPostAndSendEmail","odooPostInvoice":true,"odooSendInvoiceEmail":true,"odooEmailForceSend":true}</x:v>
       </x:c>
       <x:c r="P3" s="58" t="n">
         <x:v>60</x:v>
       </x:c>
       <x:c r="Q3" s="58" t="str">
-        <x:v>LIVE ROW DISABLED in this workbook. Use google-sheets-template-live.xlsx for live mode.</x:v>
+        <x:v>Disabled in sandbox workbook</x:v>
       </x:c>
-      <x:c r="R3" s="55"/>
-      <x:c r="S3" s="55"/>
-      <x:c r="T3" s="55"/>
-      <x:c r="U3" s="55"/>
-      <x:c r="V3" s="55"/>
-      <x:c r="W3" s="55"/>
-      <x:c r="X3" s="55"/>
-      <x:c r="Y3" s="55"/>
-      <x:c r="Z3" s="55"/>
+      <x:c r="R3" s="55" t="str">
+        <x:v>odoo-production</x:v>
+      </x:c>
+      <x:c r="S3" s="55" t="str">
+        <x:v>DISABLED_USER</x:v>
+      </x:c>
+      <x:c r="T3" s="55" t="str"/>
+      <x:c r="U3" s="72" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="V3" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="W3" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="X3" s="55" t="str"/>
+      <x:c r="Y3" s="55" t="str"/>
+      <x:c r="Z3" s="55" t="str"/>
+      <x:c r="AA3" t="str"/>
+      <x:c r="AB3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AC3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AD3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE3" t="str"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="55"/>
@@ -11930,22 +12105,36 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="57" t="str">
+      <x:c r="A1" s="75" t="str">
         <x:v>Email</x:v>
       </x:c>
-      <x:c r="B1" s="57" t="str">
+      <x:c r="B1" s="75" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="C1" s="75" t="str">
         <x:v>Name</x:v>
       </x:c>
-      <x:c r="C1" s="57" t="str">
+      <x:c r="D1" s="80" t="str">
         <x:v>Address</x:v>
       </x:c>
-      <x:c r="D1" s="55"/>
-      <x:c r="E1" s="55"/>
-      <x:c r="F1" s="55"/>
-      <x:c r="G1" s="55"/>
-      <x:c r="H1" s="55"/>
-      <x:c r="I1" s="55"/>
-      <x:c r="J1" s="55"/>
+      <x:c r="E1" s="80" t="str">
+        <x:v>Job_ID</x:v>
+      </x:c>
+      <x:c r="F1" s="80" t="str">
+        <x:v>Campaign_ID</x:v>
+      </x:c>
+      <x:c r="G1" s="80" t="str">
+        <x:v>Attempt_Count</x:v>
+      </x:c>
+      <x:c r="H1" s="80" t="str">
+        <x:v>Last_Account</x:v>
+      </x:c>
+      <x:c r="I1" s="80" t="str">
+        <x:v>Last_Error</x:v>
+      </x:c>
+      <x:c r="J1" s="80" t="str">
+        <x:v>Updated_At</x:v>
+      </x:c>
       <x:c r="K1" s="55"/>
       <x:c r="L1" s="55"/>
       <x:c r="M1" s="55"/>
@@ -11965,19 +12154,25 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="67" t="str">
-        <x:v>victorsteele428@gmail.com</x:v>
+        <x:v>customer@example.com</x:v>
       </x:c>
       <x:c r="B2" s="70" t="str">
-        <x:v>Victor Steele</x:v>
+        <x:v>PENDING</x:v>
       </x:c>
-      <x:c r="C2" s="70" t="str"/>
-      <x:c r="D2" s="55"/>
-      <x:c r="E2" s="55"/>
-      <x:c r="F2" s="55"/>
-      <x:c r="G2" s="55"/>
-      <x:c r="H2" s="55"/>
-      <x:c r="I2" s="55"/>
-      <x:c r="J2" s="55"/>
+      <x:c r="C2" s="70" t="str">
+        <x:v>Customer Example</x:v>
+      </x:c>
+      <x:c r="D2" s="55" t="str"/>
+      <x:c r="E2" s="55" t="str"/>
+      <x:c r="F2" s="55" t="str">
+        <x:v>sandbox-campaign-001</x:v>
+      </x:c>
+      <x:c r="G2" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H2" s="55" t="str"/>
+      <x:c r="I2" s="55" t="str"/>
+      <x:c r="J2" s="55" t="str"/>
       <x:c r="K2" s="55"/>
       <x:c r="L2" s="55"/>
       <x:c r="M2" s="55"/>
@@ -11999,15 +12194,21 @@
       <x:c r="A3" s="67" t="str">
         <x:v>customer2@example.com</x:v>
       </x:c>
-      <x:c r="B3" s="70" t="str"/>
+      <x:c r="B3" s="70" t="str">
+        <x:v>PENDING</x:v>
+      </x:c>
       <x:c r="C3" s="70" t="str"/>
-      <x:c r="D3" s="55"/>
-      <x:c r="E3" s="55"/>
-      <x:c r="F3" s="55"/>
-      <x:c r="G3" s="55"/>
-      <x:c r="H3" s="55"/>
-      <x:c r="I3" s="55"/>
-      <x:c r="J3" s="55"/>
+      <x:c r="D3" s="55" t="str"/>
+      <x:c r="E3" s="55" t="str"/>
+      <x:c r="F3" s="55" t="str">
+        <x:v>sandbox-campaign-001</x:v>
+      </x:c>
+      <x:c r="G3" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H3" s="55" t="str"/>
+      <x:c r="I3" s="55" t="str"/>
+      <x:c r="J3" s="55" t="str"/>
       <x:c r="K3" s="55"/>
       <x:c r="L3" s="55"/>
       <x:c r="M3" s="55"/>
@@ -12029,15 +12230,21 @@
       <x:c r="A4" s="67" t="str">
         <x:v>customer3@example.com</x:v>
       </x:c>
-      <x:c r="B4" s="70" t="str"/>
+      <x:c r="B4" s="70" t="str">
+        <x:v>PENDING</x:v>
+      </x:c>
       <x:c r="C4" s="70" t="str"/>
-      <x:c r="D4" s="55"/>
-      <x:c r="E4" s="55"/>
-      <x:c r="F4" s="55"/>
-      <x:c r="G4" s="55"/>
-      <x:c r="H4" s="55"/>
-      <x:c r="I4" s="55"/>
-      <x:c r="J4" s="55"/>
+      <x:c r="D4" s="55" t="str"/>
+      <x:c r="E4" s="55" t="str"/>
+      <x:c r="F4" s="55" t="str">
+        <x:v>sandbox-campaign-001</x:v>
+      </x:c>
+      <x:c r="G4" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H4" s="55" t="str"/>
+      <x:c r="I4" s="55" t="str"/>
+      <x:c r="J4" s="55" t="str"/>
       <x:c r="K4" s="55"/>
       <x:c r="L4" s="55"/>
       <x:c r="M4" s="55"/>
@@ -17584,197 +17791,230 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="50" customHeight="1">
-      <x:c r="A1" s="57" t="str">
+      <x:c r="A1" s="75" t="str">
         <x:v>writeback_key</x:v>
       </x:c>
-      <x:c r="B1" s="57" t="str">
+      <x:c r="B1" s="75" t="str">
         <x:v>writeback_action</x:v>
       </x:c>
-      <x:c r="C1" s="57" t="str">
+      <x:c r="C1" s="75" t="str">
         <x:v>writeback_target</x:v>
       </x:c>
-      <x:c r="D1" s="57" t="str">
+      <x:c r="D1" s="75" t="str">
         <x:v>key_mode</x:v>
       </x:c>
-      <x:c r="E1" s="57" t="str">
+      <x:c r="E1" s="75" t="str">
         <x:v>request_id</x:v>
       </x:c>
-      <x:c r="F1" s="57" t="str">
+      <x:c r="F1" s="75" t="str">
         <x:v>transaction_id</x:v>
       </x:c>
-      <x:c r="G1" s="57" t="str">
+      <x:c r="G1" s="75" t="str">
         <x:v>idempotency_key</x:v>
       </x:c>
-      <x:c r="H1" s="57" t="str">
+      <x:c r="H1" s="75" t="str">
+        <x:v>job_id</x:v>
+      </x:c>
+      <x:c r="I1" s="75" t="str">
+        <x:v>campaign_id</x:v>
+      </x:c>
+      <x:c r="J1" s="75" t="str">
         <x:v>provider_id</x:v>
       </x:c>
-      <x:c r="I1" s="57" t="str">
+      <x:c r="K1" s="75" t="str">
         <x:v>profile_id</x:v>
       </x:c>
-      <x:c r="J1" s="57" t="str">
+      <x:c r="L1" s="75" t="str">
         <x:v>account_id</x:v>
       </x:c>
-      <x:c r="K1" s="57" t="str">
+      <x:c r="M1" s="75" t="str">
         <x:v>action_id</x:v>
       </x:c>
-      <x:c r="L1" s="57" t="str">
+      <x:c r="N1" s="75" t="str">
         <x:v>worker_id</x:v>
       </x:c>
-      <x:c r="M1" s="57" t="str">
+      <x:c r="O1" s="75" t="str">
         <x:v>recipient_email</x:v>
       </x:c>
-      <x:c r="N1" s="57" t="str">
+      <x:c r="P1" s="75" t="str">
         <x:v>workflow_state</x:v>
       </x:c>
-      <x:c r="O1" s="57" t="str">
+      <x:c r="Q1" s="75" t="str">
         <x:v>result</x:v>
       </x:c>
-      <x:c r="P1" s="57" t="str">
+      <x:c r="R1" s="75" t="str">
         <x:v>invoice_status</x:v>
       </x:c>
-      <x:c r="Q1" s="57" t="str">
+      <x:c r="S1" s="75" t="str">
         <x:v>provider_status</x:v>
       </x:c>
-      <x:c r="R1" s="57" t="str">
+      <x:c r="T1" s="75" t="str">
         <x:v>transport_status</x:v>
       </x:c>
-      <x:c r="S1" s="57" t="str">
+      <x:c r="U1" s="75" t="str">
         <x:v>provider_customer_id</x:v>
       </x:c>
-      <x:c r="T1" s="57" t="str">
+      <x:c r="V1" s="75" t="str">
         <x:v>customer_status</x:v>
       </x:c>
-      <x:c r="U1" s="57" t="str">
+      <x:c r="W1" s="75" t="str">
         <x:v>post_status</x:v>
       </x:c>
-      <x:c r="V1" s="57" t="str">
+      <x:c r="X1" s="75" t="str">
         <x:v>email_send_requested</x:v>
       </x:c>
-      <x:c r="W1" s="57" t="str">
+      <x:c r="Y1" s="75" t="str">
         <x:v>email_send_status</x:v>
       </x:c>
-      <x:c r="X1" s="57" t="str">
+      <x:c r="Z1" s="75" t="str">
         <x:v>email_send_method</x:v>
       </x:c>
-      <x:c r="Y1" s="57" t="str">
+      <x:c r="AA1" s="82" t="str">
         <x:v>email_error_message</x:v>
       </x:c>
-      <x:c r="Z1" s="57" t="str">
+      <x:c r="AB1" s="82" t="str">
+        <x:v>email_evidence</x:v>
+      </x:c>
+      <x:c r="AC1" s="82" t="str">
+        <x:v>lifecycle_outcome</x:v>
+      </x:c>
+      <x:c r="AD1" s="82" t="str">
+        <x:v>lifecycle_failed_step</x:v>
+      </x:c>
+      <x:c r="AE1" s="82" t="str">
+        <x:v>lifecycle_checkpoint</x:v>
+      </x:c>
+      <x:c r="AF1" s="82" t="str">
+        <x:v>retry_resume_stage</x:v>
+      </x:c>
+      <x:c r="AG1" s="82" t="str">
+        <x:v>retry_resume</x:v>
+      </x:c>
+      <x:c r="AH1" s="82" t="str">
         <x:v>provider_invoice_id</x:v>
       </x:c>
-      <x:c r="AA1" s="20" t="str">
+      <x:c r="AI1" s="82" t="str">
         <x:v>invoice_number</x:v>
       </x:c>
-      <x:c r="AB1" s="20" t="str">
+      <x:c r="AJ1" s="82" t="str">
         <x:v>invoice_url</x:v>
       </x:c>
-      <x:c r="AC1" s="20" t="str">
+      <x:c r="AK1" s="82" t="str">
         <x:v>pdf_url</x:v>
       </x:c>
-      <x:c r="AD1" s="20" t="str">
+      <x:c r="AL1" s="82" t="str">
         <x:v>http_status</x:v>
       </x:c>
-      <x:c r="AE1" s="20" t="str">
+      <x:c r="AM1" s="82" t="str">
         <x:v>error_type</x:v>
       </x:c>
-      <x:c r="AF1" s="20" t="str">
+      <x:c r="AN1" s="82" t="str">
         <x:v>error_category</x:v>
       </x:c>
-      <x:c r="AG1" s="20" t="str">
+      <x:c r="AO1" s="82" t="str">
         <x:v>error_severity</x:v>
       </x:c>
-      <x:c r="AH1" s="20" t="str">
+      <x:c r="AP1" s="82" t="str">
         <x:v>error_code</x:v>
       </x:c>
-      <x:c r="AI1" s="20" t="str">
+      <x:c r="AQ1" s="82" t="str">
         <x:v>error_message</x:v>
       </x:c>
-      <x:c r="AJ1" s="20" t="str">
+      <x:c r="AR1" s="82" t="str">
         <x:v>retry_scheduled</x:v>
       </x:c>
-      <x:c r="AK1" s="20" t="str">
+      <x:c r="AS1" s="82" t="str">
         <x:v>retry_count</x:v>
       </x:c>
-      <x:c r="AL1" s="20" t="str">
+      <x:c r="AT1" s="82" t="str">
         <x:v>retry_delay_seconds</x:v>
       </x:c>
-      <x:c r="AM1" s="20" t="str">
+      <x:c r="AU1" s="82" t="str">
         <x:v>retry_decision_source</x:v>
       </x:c>
-      <x:c r="AN1" s="20" t="str">
+      <x:c r="AV1" s="82" t="str">
         <x:v>retry_decision_reason</x:v>
       </x:c>
-      <x:c r="AO1" s="20" t="str">
+      <x:c r="AW1" s="82" t="str">
         <x:v>retry_after_seconds</x:v>
       </x:c>
-      <x:c r="AP1" s="20" t="str">
+      <x:c r="AX1" s="82" t="str">
         <x:v>retry_delay_hint_seconds</x:v>
       </x:c>
-      <x:c r="AQ1" s="20" t="str">
+      <x:c r="AY1" s="82" t="str">
         <x:v>next_retry_at</x:v>
       </x:c>
-      <x:c r="AR1" s="20" t="str">
+      <x:c r="AZ1" s="82" t="str">
         <x:v>lifecycle_mode</x:v>
       </x:c>
-      <x:c r="AS1" s="20" t="str">
+      <x:c r="BA1" s="82" t="str">
         <x:v>lifecycle_steps</x:v>
       </x:c>
-      <x:c r="AT1" s="20" t="str">
+      <x:c r="BB1" s="82" t="str">
         <x:v>provider_recipe_id</x:v>
       </x:c>
-      <x:c r="AU1" s="20" t="str">
+      <x:c r="BC1" s="82" t="str">
         <x:v>preset_self_check_mode</x:v>
       </x:c>
-      <x:c r="AV1" s="20" t="str">
+      <x:c r="BD1" s="82" t="str">
         <x:v>preset_self_check_approved</x:v>
       </x:c>
-      <x:c r="AW1" s="20" t="str">
+      <x:c r="BE1" s="82" t="str">
         <x:v>preset_self_check</x:v>
       </x:c>
-      <x:c r="AX1" s="20" t="str">
+      <x:c r="BF1" s="82" t="str">
         <x:v>activation_mode</x:v>
       </x:c>
-      <x:c r="AY1" s="20" t="str">
+      <x:c r="BG1" s="82" t="str">
         <x:v>activation_approved</x:v>
       </x:c>
-      <x:c r="AZ1" s="20" t="str">
+      <x:c r="BH1" s="82" t="str">
         <x:v>activation_safety</x:v>
       </x:c>
-      <x:c r="BA1" s="20" t="str">
+      <x:c r="BI1" s="82" t="str">
         <x:v>bulk_run_id</x:v>
       </x:c>
-      <x:c r="BB1" s="20" t="str">
+      <x:c r="BJ1" s="82" t="str">
         <x:v>bulk_item_number</x:v>
       </x:c>
-      <x:c r="BC1" s="20" t="str">
+      <x:c r="BK1" s="82" t="str">
         <x:v>bulk_total_items</x:v>
       </x:c>
-      <x:c r="BD1" s="20" t="str">
+      <x:c r="BL1" s="82" t="str">
         <x:v>bulk_decision</x:v>
       </x:c>
-      <x:c r="BE1" s="20" t="str">
+      <x:c r="BM1" s="81" t="str">
         <x:v>bulk_safety</x:v>
       </x:c>
-      <x:c r="BF1" s="20" t="str">
+      <x:c r="BN1" s="81" t="str">
         <x:v>bulk_summary</x:v>
       </x:c>
-      <x:c r="BG1" s="20" t="str">
+      <x:c r="BO1" s="81" t="str">
         <x:v>retryable_by_policy</x:v>
       </x:c>
-      <x:c r="BH1" s="20" t="str">
+      <x:c r="BP1" s="81" t="str">
         <x:v>non_retryable_by_policy</x:v>
       </x:c>
-      <x:c r="BI1" s="20" t="str">
+      <x:c r="BQ1" s="81" t="str">
         <x:v>duplicate_prevention</x:v>
       </x:c>
-      <x:c r="BJ1" s="20" t="str">
+      <x:c r="BR1" s="81" t="str">
         <x:v>checked_at</x:v>
       </x:c>
-      <x:c r="BK1" s="20" t="str">
+      <x:c r="BS1" s="81" t="str">
         <x:v>managed_at</x:v>
       </x:c>
-      <x:c r="BL1" s="20" t="str">
+      <x:c r="BT1" s="81" t="str">
         <x:v>updated_at</x:v>
+      </x:c>
+      <x:c r="BU1" s="81" t="str">
+        <x:v>failover_scheduled</x:v>
+      </x:c>
+      <x:c r="BV1" s="81" t="str">
+        <x:v>recipient_status</x:v>
+      </x:c>
+      <x:c r="BW1" s="81" t="str">
+        <x:v>provider_operational_status</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -34795,7 +35035,7 @@
         <x:v>Odoo base domain without trailing slash</x:v>
       </x:c>
       <x:c r="E2" s="58" t="str">
-        <x:v>https://apple-zone1.odoo.com</x:v>
+        <x:v>https://YOUR-SUBDOMAIN.odoo.com</x:v>
       </x:c>
       <x:c r="F2" s="55"/>
       <x:c r="G2" s="55"/>
@@ -34947,7 +35187,7 @@
         <x:v>Exact Odoo database technical name</x:v>
       </x:c>
       <x:c r="E6" s="58" t="str">
-        <x:v>apple-zone1</x:v>
+        <x:v>YOUR_ODOO_DATABASE</x:v>
       </x:c>
       <x:c r="F6" s="55"/>
       <x:c r="G6" s="55"/>
@@ -40446,4 +40686,155 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="81" t="str">
+        <x:v>Job_ID</x:v>
+      </x:c>
+      <x:c r="B1" s="81" t="str">
+        <x:v>Campaign_ID</x:v>
+      </x:c>
+      <x:c r="C1" s="81" t="str">
+        <x:v>Recipient_Email</x:v>
+      </x:c>
+      <x:c r="D1" s="81" t="str">
+        <x:v>Original_Profile_ID</x:v>
+      </x:c>
+      <x:c r="E1" s="81" t="str">
+        <x:v>Current_Profile_ID</x:v>
+      </x:c>
+      <x:c r="F1" s="81" t="str">
+        <x:v>Attempted_Profile_IDs</x:v>
+      </x:c>
+      <x:c r="G1" s="81" t="str">
+        <x:v>Failover_Group</x:v>
+      </x:c>
+      <x:c r="H1" s="81" t="str">
+        <x:v>Side_Effect_Stage</x:v>
+      </x:c>
+      <x:c r="I1" s="81" t="str">
+        <x:v>Required_Profile_ID</x:v>
+      </x:c>
+      <x:c r="J1" s="81" t="str">
+        <x:v>Provider_Invoice_ID</x:v>
+      </x:c>
+      <x:c r="K1" s="81" t="str">
+        <x:v>Lifecycle_Checkpoint</x:v>
+      </x:c>
+      <x:c r="L1" s="81" t="str">
+        <x:v>Resume_Stage</x:v>
+      </x:c>
+      <x:c r="M1" s="81" t="str">
+        <x:v>Retry_Count</x:v>
+      </x:c>
+      <x:c r="N1" s="81" t="str">
+        <x:v>Failover_Count</x:v>
+      </x:c>
+      <x:c r="O1" s="81" t="str">
+        <x:v>Next_Retry_At</x:v>
+      </x:c>
+      <x:c r="P1" s="81" t="str">
+        <x:v>Last_Error_Type</x:v>
+      </x:c>
+      <x:c r="Q1" s="81" t="str">
+        <x:v>Last_Error</x:v>
+      </x:c>
+      <x:c r="R1" s="81" t="str">
+        <x:v>Queue_Status</x:v>
+      </x:c>
+      <x:c r="S1" s="81" t="str">
+        <x:v>Updated_At</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="81" t="str">
+        <x:v>Report_Key</x:v>
+      </x:c>
+      <x:c r="B1" s="81" t="str">
+        <x:v>Campaign_ID</x:v>
+      </x:c>
+      <x:c r="C1" s="81" t="str">
+        <x:v>Provider</x:v>
+      </x:c>
+      <x:c r="D1" s="81" t="str">
+        <x:v>Account_ID</x:v>
+      </x:c>
+      <x:c r="E1" s="81" t="str">
+        <x:v>Account_Name</x:v>
+      </x:c>
+      <x:c r="F1" s="81" t="str">
+        <x:v>Profile_ID</x:v>
+      </x:c>
+      <x:c r="G1" s="81" t="str">
+        <x:v>Current_Status</x:v>
+      </x:c>
+      <x:c r="H1" s="81" t="str">
+        <x:v>Enabled</x:v>
+      </x:c>
+      <x:c r="I1" s="81" t="str">
+        <x:v>Allocated</x:v>
+      </x:c>
+      <x:c r="J1" s="81" t="str">
+        <x:v>Attempted</x:v>
+      </x:c>
+      <x:c r="K1" s="81" t="str">
+        <x:v>Succeeded</x:v>
+      </x:c>
+      <x:c r="L1" s="81" t="str">
+        <x:v>Email_Sent</x:v>
+      </x:c>
+      <x:c r="M1" s="81" t="str">
+        <x:v>Email_Queued</x:v>
+      </x:c>
+      <x:c r="N1" s="81" t="str">
+        <x:v>Failed</x:v>
+      </x:c>
+      <x:c r="O1" s="81" t="str">
+        <x:v>Retried</x:v>
+      </x:c>
+      <x:c r="P1" s="81" t="str">
+        <x:v>Failover_Count</x:v>
+      </x:c>
+      <x:c r="Q1" s="81" t="str">
+        <x:v>Failover_From</x:v>
+      </x:c>
+      <x:c r="R1" s="81" t="str">
+        <x:v>Failover_To</x:v>
+      </x:c>
+      <x:c r="S1" s="81" t="str">
+        <x:v>Auto_Disabled</x:v>
+      </x:c>
+      <x:c r="T1" s="81" t="str">
+        <x:v>Disabled_Reason</x:v>
+      </x:c>
+      <x:c r="U1" s="81" t="str">
+        <x:v>Last_Error_Type</x:v>
+      </x:c>
+      <x:c r="V1" s="81" t="str">
+        <x:v>Last_Error</x:v>
+      </x:c>
+      <x:c r="W1" s="81" t="str">
+        <x:v>Last_Used_At</x:v>
+      </x:c>
+      <x:c r="X1" s="81" t="str">
+        <x:v>Updated_At</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>